<commit_message>
Fix S/O, D/O, W/O label overlap with father's name on certificates
The GD Goenka certificate template's parent-name label was changed from
"Son of" to "S/O, D/O, W/O" to cover daughters and married candidates,
but the longer label text now overlapped the FATHER_NAME value's default
x-position (calibrated for the shorter "Son of"). Shift the default
FATHER_NAME x from 135 to 160 so the value renders clear of the label,
and update the bundled sample template files to match.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/samples/Candidate_Import_Template.xlsx
+++ b/templates/samples/Candidate_Import_Template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0FE560C-7548-41F3-9E0F-98F585A0A0A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDFB6013-BCC6-4873-8481-A9545A5CA1D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="25">
   <si>
     <t>Certificate No</t>
   </si>
@@ -53,73 +53,43 @@
     <t>Remarks</t>
   </si>
   <si>
-    <t>Diploma in Computer Applications</t>
-  </si>
-  <si>
-    <t>6 Months</t>
-  </si>
-  <si>
     <t>A+</t>
   </si>
   <si>
     <t>Completed with distinction</t>
   </si>
   <si>
-    <t>Diploma in Financial Accounting</t>
-  </si>
-  <si>
-    <t>3 Months</t>
-  </si>
-  <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>Certificate in Tally &amp; GST</t>
-  </si>
-  <si>
-    <t>2 Months</t>
-  </si>
-  <si>
-    <t>B+</t>
-  </si>
-  <si>
-    <t xml:space="preserve">abdul </t>
-  </si>
-  <si>
-    <t>Rakesh Sharme</t>
-  </si>
-  <si>
-    <t>Suresh Verme</t>
-  </si>
-  <si>
-    <t>NCEVT/2026/010</t>
-  </si>
-  <si>
-    <t>ENR-2026-0010</t>
-  </si>
-  <si>
-    <t>NCEVT/2026/011</t>
-  </si>
-  <si>
-    <t>ENR-2026-0011</t>
-  </si>
-  <si>
-    <t>NCEVT/2026/012</t>
-  </si>
-  <si>
-    <t>ENR-2026-0012</t>
-  </si>
-  <si>
-    <t>Test User 1</t>
-  </si>
-  <si>
-    <t>Test User 2</t>
-  </si>
-  <si>
-    <t>Test user 3</t>
+    <t>Raja</t>
+  </si>
+  <si>
+    <t>S/o Naresh</t>
+  </si>
+  <si>
+    <t>Retail Sales Assistant</t>
+  </si>
+  <si>
+    <t>60 Days</t>
+  </si>
+  <si>
+    <t>23/07/2026</t>
+  </si>
+  <si>
+    <t>Prince</t>
+  </si>
+  <si>
+    <t>S/o Puran singh</t>
+  </si>
+  <si>
+    <t>TESTD00300</t>
+  </si>
+  <si>
+    <t>TESTD00301</t>
+  </si>
+  <si>
+    <t>TEST0426300</t>
+  </si>
+  <si>
+    <t>TEST0426301</t>
   </si>
 </sst>
 </file>
@@ -523,7 +493,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="3" width="20" customWidth="1"/>
@@ -575,57 +545,57 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="B2" t="s">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="C2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" s="1">
+        <v>39503</v>
+      </c>
+      <c r="E2" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="1">
-        <v>46218</v>
-      </c>
-      <c r="E2" t="s">
-        <v>27</v>
-      </c>
       <c r="F2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" t="s">
         <v>12</v>
       </c>
-      <c r="G2" t="s">
+      <c r="I2" s="1">
+        <v>46330</v>
+      </c>
+      <c r="J2" s="1">
+        <v>46301</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="L2" t="s">
         <v>13</v>
-      </c>
-      <c r="H2" t="s">
-        <v>14</v>
-      </c>
-      <c r="I2" s="1">
-        <v>46027</v>
-      </c>
-      <c r="J2" s="1">
-        <v>46203</v>
-      </c>
-      <c r="K2" s="1">
-        <v>46213</v>
-      </c>
-      <c r="L2" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="B3" t="s">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="C3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" s="1">
+        <v>39460</v>
+      </c>
+      <c r="E3" t="s">
         <v>24</v>
-      </c>
-      <c r="D3" s="1">
-        <v>37723</v>
-      </c>
-      <c r="E3" t="s">
-        <v>29</v>
       </c>
       <c r="F3" t="s">
         <v>16</v>
@@ -634,57 +604,16 @@
         <v>17</v>
       </c>
       <c r="H3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I3" s="1">
+        <v>46330</v>
+      </c>
+      <c r="J3" s="1">
+        <v>46301</v>
+      </c>
+      <c r="K3" s="1" t="s">
         <v>18</v>
-      </c>
-      <c r="I3" s="1">
-        <v>46054</v>
-      </c>
-      <c r="J3" s="1">
-        <v>46142</v>
-      </c>
-      <c r="K3" s="1">
-        <v>46147</v>
-      </c>
-      <c r="L3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D4" s="1">
-        <v>37520</v>
-      </c>
-      <c r="E4" t="s">
-        <v>31</v>
-      </c>
-      <c r="F4" t="s">
-        <v>20</v>
-      </c>
-      <c r="G4" t="s">
-        <v>21</v>
-      </c>
-      <c r="H4" t="s">
-        <v>22</v>
-      </c>
-      <c r="I4" s="1">
-        <v>46091</v>
-      </c>
-      <c r="J4" s="1">
-        <v>46152</v>
-      </c>
-      <c r="K4" s="1">
-        <v>46157</v>
-      </c>
-      <c r="L4" t="s">
-        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>